<commit_message>
Audit phase 3: landing page
Hero: one explanatory sentence, one question box, one primary action; the blurred record
background, the lens and the example chips are gone. The approval sentence appears once, in the
hero. New computed price strip (5 companies, 100 posts on X) from the shared estimate. Merged
sections «إزاي بيشتغل وإيه اللي بتدفعه» and «إيه اللي ممكن تطلبه». The sample is labelled
«نموذج توضيحي» and carries no link, e-mail or example.com. Short FAQ (price, legality, partial
delivery, top-up) using the pricing page's own answers. One closing action; the footer is unchanged.
Home route: 16.7 kB / 244 kB -> 8.2 kB / 224 kB first load.

No price, cap or pricing-function change. No SQL.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qry3DqAaJ3VvWuiZJHYpQy
</commit_message>
<xml_diff>
--- a/public/samples/diger-sample-comments.xlsx
+++ b/public/samples/diger-sample-comments.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
   <si>
     <t>معرف السجل</t>
   </si>
@@ -31,9 +31,6 @@
     <t>عنوان الفيديو أو المنشور</t>
   </si>
   <si>
-    <t>رابط الفيديو أو المنشور</t>
-  </si>
-  <si>
     <t>معرف المصدر الأصلي</t>
   </si>
   <si>
@@ -50,9 +47,6 @@
   </si>
   <si>
     <t>فيديو تجريبي</t>
-  </si>
-  <si>
-    <t>https://example.com/demo-video</t>
   </si>
   <si>
     <t>demo_c1</t>
@@ -137,7 +131,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -148,12 +142,6 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0563C1"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
@@ -208,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -219,13 +207,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -570,7 +552,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -578,11 +560,10 @@
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
-    <col min="7" max="7" width="32" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -604,176 +585,147 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="22" customHeight="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="4" t="s">
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
+      <c r="D3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="22" customHeight="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="3" t="s">
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="D5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="22" customHeight="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="F6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="3" t="s">
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="F7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1"/>
-    <hyperlink ref="G3" r:id="rId2"/>
-    <hyperlink ref="G4" r:id="rId3"/>
-    <hyperlink ref="G5" r:id="rId4"/>
-    <hyperlink ref="G6" r:id="rId5"/>
-    <hyperlink ref="G7" r:id="rId6"/>
-  </hyperlinks>
+  <autoFilter ref="A1:G7"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>